<commit_message>
excel y los responsables
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -2081,7 +2081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" ht="72" customHeight="1">
@@ -2100,6 +2100,11 @@
           <t>51.8247, 5.8650</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>MARIA JULIA FLORES GALLEGO</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
@@ -2117,6 +2122,11 @@
           <t>48.1396, 17.1168</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Mª DEL CARMEN RUIZ DELGADO</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="86.40000000000001" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -2134,6 +2144,11 @@
           <t>59.6111, 16.5464</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ENRIQUE ARIAS ANTÚNEZ</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.6" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -2151,6 +2166,11 @@
           <t>50.0674, 19.9126</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MANUEL ÁNGEL SERRANO MARTÍN</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -2168,6 +2188,11 @@
           <t>53.1325, 23.1688</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>JESÚS SERRANO GUERRERO</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28.8" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -2185,6 +2210,11 @@
           <t>59.3710, 16.5097</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ENRIQUE ARIAS ANTÚNEZ</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -2202,6 +2232,11 @@
           <t>50.0413, 21.9990</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AURORA VIZCAÍNO BARCELÓ</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28.8" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -2219,6 +2254,11 @@
           <t>59.6111, 16.5464</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ENRIQUE ARIAS ANTÚNEZ</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.6" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -2236,6 +2276,11 @@
           <t>32.6589, -16.9246</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>VÍCTOR MANUEL LÓPEZ JAQUERO</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="57.6" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -2253,6 +2298,11 @@
           <t>46.5592, 15.6433</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>JESÚS SERRANO GUERRERO</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="57.6" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -2270,6 +2320,11 @@
           <t>63.8198, 20.3053</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GINÉS DAMIÁN MORENO VALVERDE</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="57.6" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -2287,6 +2342,11 @@
           <t>48.1396, 17.1168</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mª DEL CARMEN RUIZ DELGADO</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="43.2" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -2304,6 +2364,11 @@
           <t>46.5592, 15.6433</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>JESÚS SERRANO GUERRERO</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28.8" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -2321,6 +2386,11 @@
           <t>51.5242, -0.1330</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>JESÚS SERRANO GUERRERO</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="28.8" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -2338,6 +2408,11 @@
           <t>50.0413, 21.9990</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>AURORA VIZCAÍNO BARCELÓ</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="43.2" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -2355,6 +2430,11 @@
           <t>49.8346, 18.2820</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MANUEL ÁNGEL SERRANO MARTÍN</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="28.8" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -2372,6 +2452,11 @@
           <t>50.0413, 21.9990</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>AURORA VIZCAÍNO BARCELÓ</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="57.6" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -2387,6 +2472,11 @@
       <c r="C18" s="6" t="inlineStr">
         <is>
           <t>41.1095, 16.8817</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>JESÚS SERRANO GUERRERO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Arreglo de estadísticas y responsables
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="2025-2026" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,12 +48,6 @@
       <color theme="10"/>
       <sz val="11"/>
       <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -155,7 +149,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5432,7 +5426,6 @@
         </is>
       </c>
     </row>
-    <row r="150"/>
     <row r="151">
       <c r="O151" s="9" t="n"/>
     </row>
@@ -5846,16 +5839,21 @@
   </sheetPr>
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="11.44140625" customWidth="1" min="1" max="1"/>
+    <col width="11.44140625" customWidth="1" min="3" max="4"/>
+    <col width="11.44140625" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1" ht="72" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
+          <t>Radboud Universiteit Nijmegen</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
           <t>Países Bajos</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Radboud Universiteit Nijmegen</t>
         </is>
       </c>
       <c r="C1" s="6" t="inlineStr">
@@ -5872,12 +5870,12 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
+          <t>Comenius University in Bratislava</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
           <t>República Eslovaca</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Comenius University in Bratislava</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -5894,12 +5892,12 @@
     <row r="3" ht="86.40000000000001" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
+          <t>Mälardalen University</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
           <t>Suecia</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Mälardalen University</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -5916,12 +5914,12 @@
     <row r="4" ht="57.6" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
+          <t>AGH University of Science and Technology</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
           <t>Polonia</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>AGH University of Science and Technology</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -5938,12 +5936,12 @@
     <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
+          <t>Bialystok University of Technology</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
           <t>Polonia</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Bialystok University of Technology</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -5960,12 +5958,12 @@
     <row r="6" ht="28.8" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
+          <t>Mälardalen University</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
           <t>Suecia</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Mälardalen University</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -5982,34 +5980,29 @@
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>University of Rzeszów</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
           <t>Polonia</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>University of Rzeszów</t>
-        </is>
-      </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
           <t>50.0413, 21.9990</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>AURORA VIZCAÍNO BARCELÓ</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28.8" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
+          <t>Mälardalen University</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
           <t>Suecia</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Mälardalen University</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -6026,78 +6019,63 @@
     <row r="9" ht="57.6" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>Universidade da Madeira</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Universidade da Madeira</t>
-        </is>
-      </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
           <t>32.6589, -16.9246</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>VÍCTOR MANUEL LÓPEZ JAQUERO</t>
         </is>
       </c>
     </row>
     <row r="10" ht="57.6" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
+          <t>University of Maribor</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
           <t>Eslovenia</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>University of Maribor</t>
-        </is>
-      </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
           <t>46.5592, 15.6433</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>JESÚS SERRANO GUERRERO</t>
         </is>
       </c>
     </row>
     <row r="11" ht="57.6" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>Umea University</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
           <t>Suecia</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Umea University</t>
-        </is>
-      </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
           <t>63.8198, 20.3053</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>GINÉS DAMIÁN MORENO VALVERDE</t>
         </is>
       </c>
     </row>
     <row r="12" ht="57.6" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
+          <t>Comenius University in Bratislava</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
           <t>República Eslovaca</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Comenius University in Bratislava</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -6114,144 +6092,114 @@
     <row r="13" ht="43.2" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>University of Maribor</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
           <t>Eslovenia</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>University of Maribor</t>
-        </is>
-      </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
           <t>46.5592, 15.6433</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>JESÚS SERRANO GUERRERO</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28.8" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
+          <t>London University</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
           <t>Reino Unido</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>London University</t>
-        </is>
-      </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
           <t>51.5242, -0.1330</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>JESÚS SERRANO GUERRERO</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28.8" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>University of Rzeszów</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
           <t>Polonia</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>University of Rzeszów</t>
-        </is>
-      </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
           <t>50.0413, 21.9990</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>AURORA VIZCAÍNO BARCELÓ</t>
         </is>
       </c>
     </row>
     <row r="16" ht="43.2" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>Technical University of Ostrava</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>República Checa</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Technical University of Ostrava</t>
-        </is>
-      </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
           <t>49.8346, 18.2820</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MANUEL ÁNGEL SERRANO MARTÍN</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28.8" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>University of Rzeszów</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
           <t>Polonia</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>University of Rzeszów</t>
-        </is>
-      </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
           <t>50.0413, 21.9990</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>AURORA VIZCAÍNO BARCELÓ</t>
         </is>
       </c>
     </row>
     <row r="18" ht="57.6" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
+          <t>Università degli Studi di Bari Aldo Moro</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
           <t>Italia</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Università degli Studi di Bari Aldo Moro</t>
-        </is>
-      </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
           <t>41.1095, 16.8817</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>JESÚS SERRANO GUERRERO</t>
         </is>
       </c>
     </row>
     <row r="19" ht="43.2" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
+          <t>University of Bari Aldo Moro</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
           <t>Italia</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>University of Bari Aldo Moro</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">

</xml_diff>

<commit_message>
actualización del pages con la estructura de erasmus out
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="600" firstSheet="1" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="2025-2026" sheetId="1" state="visible" r:id="rId1"/>
@@ -620,7 +620,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>MARIA JULIA FLORES GALLEGO</t>
+          <t>responsable 1</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Mª DEL CARMEN RUIZ DELGADO</t>
+          <t>responsable 2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ENRIQUE ARIAS ANTÚNEZ</t>
+          <t>responsable 3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MANUEL ÁNGEL SERRANO MARTÍN</t>
+          <t>responsable 4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>JESÚS SERRANO GUERRERO</t>
+          <t>responsable 5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MARCELA FABIANA GENERO BOCCO</t>
+          <t>responsable 6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AURORA VIZCAÍNO BARCELÓ</t>
+          <t>responsable 7</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MARIA JULIA FLORES GALLEGO</t>
+          <t>responsable 1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>VÍCTOR MANUEL LÓPEZ JAQUERO</t>
+          <t>responsable 8</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>JESÚS SERRANO GUERRERO</t>
+          <t>responsable 5</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>GINÉS DAMIÁN MORENO VALVERDE</t>
+          <t>responsable 9</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Mª DEL CARMEN RUIZ DELGADO</t>
+          <t>responsable 2</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>JESÚS SERRANO GUERRERO</t>
+          <t>responsable 5</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>JESÚS SERRANO GUERRERO</t>
+          <t>responsable 5</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>AURORA VIZCAÍNO BARCELÓ</t>
+          <t>responsable 7</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>MANUEL ÁNGEL SERRANO MARTÍN</t>
+          <t>responsable 4</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>AURORA VIZCAÍNO BARCELÓ</t>
+          <t>responsable 7</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>JESÚS SERRANO GUERRERO</t>
+          <t>responsable 5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>JESÚS SERRANO GUERRERO</t>
+          <t>responsable 5</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5863,7 +5863,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>MARIA JULIA FLORES GALLEGO</t>
+          <t>responsable 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
comentado parte de cloudflare y arreglado problema con el botón de escondido del sidebar
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5760" yWindow="0" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="2025-2026" sheetId="1" state="visible" r:id="rId1"/>
@@ -676,11 +676,6 @@
       <c r="F3" t="n">
         <v>5</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>responsable 2</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>https://pedro-la.com</t>
@@ -739,11 +734,6 @@
       <c r="F4" t="n">
         <v>2</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>responsable 3</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>https://anna-la.com</t>
@@ -802,11 +792,6 @@
       <c r="F5" t="n">
         <v>9</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>responsable 4</t>
-        </is>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>https://sofia-la.com</t>
@@ -865,11 +850,6 @@
       <c r="F6" t="n">
         <v>9</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>responsable 5</t>
-        </is>
-      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>https://jean-la.com</t>
@@ -925,11 +905,6 @@
       <c r="E7" t="n">
         <v>3</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>responsable 6</t>
-        </is>
-      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>https://elena-la.ccom</t>
@@ -988,11 +963,6 @@
       <c r="F8" t="n">
         <v>5</v>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>responsable 7</t>
-        </is>
-      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>https://marta-la.com</t>
@@ -1051,11 +1021,6 @@
       <c r="F9" t="n">
         <v>9</v>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>responsable 1</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>https://radboud.nl/pablo</t>
@@ -1109,11 +1074,6 @@
       <c r="F10" t="n">
         <v>6</v>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>responsable 8</t>
-        </is>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>https://carla-la.com</t>
@@ -1172,11 +1132,6 @@
       <c r="F11" t="n">
         <v>5</v>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>responsable 5</t>
-        </is>
-      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>https://diego-la.com</t>
@@ -1235,11 +1190,6 @@
       <c r="F12" t="n">
         <v>6</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>responsable 9</t>
-        </is>
-      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>https://valentina-la.com</t>
@@ -1298,11 +1248,6 @@
       <c r="F13" t="n">
         <v>5</v>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>responsable 2</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>https://daniel-la.com</t>
@@ -1361,11 +1306,6 @@
       <c r="F14" t="n">
         <v>5</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>responsable 5</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>https://um.si/ana</t>
@@ -1413,11 +1353,6 @@
           <t>carla.oliveira@uclm.es</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>responsable 5</t>
-        </is>
-      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://carla-la.com</t>
@@ -1471,11 +1406,6 @@
       <c r="F16" t="n">
         <v>5</v>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>responsable 7</t>
-        </is>
-      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>https://ines-la.com</t>
@@ -1534,11 +1464,6 @@
       <c r="F17" t="n">
         <v>5</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>responsable 4</t>
-        </is>
-      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>https://samuel-la.com</t>
@@ -1597,11 +1522,6 @@
       <c r="F18" t="n">
         <v>5</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>responsable 7</t>
-        </is>
-      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>https://beatriz-la.com</t>
@@ -1664,11 +1584,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>responsable 5</t>
-        </is>
-      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>TFG_MariaPicazoSanchez (2).pdf</t>
@@ -1722,11 +1637,6 @@
       <c r="F20" t="n">
         <v>5</v>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>responsable 5</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>https://ku.lt/nuria</t>
@@ -1764,6 +1674,11 @@
           <t>Ape2. 20</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>responsable 2</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
@@ -2142,6 +2057,11 @@
           <t>Ape2. 34</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>responsable 3</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
@@ -2736,6 +2656,11 @@
           <t>Ape2. 56</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>responsable 4</t>
+        </is>
+      </c>
       <c r="J57" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3504,6 +3429,11 @@
           <t>Ape2. 80</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>responsable 5</t>
+        </is>
+      </c>
       <c r="J81" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
@@ -3774,6 +3704,11 @@
           <t>Ape2. 90</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>repsonsable 6</t>
+        </is>
+      </c>
       <c r="J91" t="inlineStr">
         <is>
           <t>London University</t>
@@ -4222,6 +4157,11 @@
           <t>Ape2. 104</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>responsable 7</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
@@ -4713,6 +4653,11 @@
           <t>Alu122@correo.com</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>responsable 8</t>
+        </is>
+      </c>
       <c r="J123" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
@@ -5278,6 +5223,11 @@
       <c r="C144" t="inlineStr">
         <is>
           <t>Ape2. 143</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>responsable 9</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -5858,6 +5808,11 @@
           <t>48.1396, 17.1168</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>responsable 2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="86.40000000000001" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -5875,6 +5830,11 @@
           <t>59.6111, 16.5464</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>responsable 8</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.6" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -5892,6 +5852,11 @@
           <t>50.0674, 19.9126</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>responsable 5</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -5926,6 +5891,11 @@
           <t>59.3710, 16.5097</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>responsable 8</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -5943,6 +5913,11 @@
           <t>50.0413, 21.9990</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>responsable 3</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28.8" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -5960,6 +5935,11 @@
           <t>59.6111, 16.5464</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>responsable 8</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.6" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -5977,6 +5957,11 @@
           <t>32.6589, -16.9246</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>responsable 7</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="57.6" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -6028,6 +6013,11 @@
           <t>48.1396, 17.1168</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>responsable 2</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="43.2" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -6062,6 +6052,11 @@
           <t>51.5242, -0.1330</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>repsonsable 6</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="28.8" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -6079,6 +6074,11 @@
           <t>50.0413, 21.9990</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>responsable 3</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="43.2" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -6113,6 +6113,11 @@
           <t>50.0413, 21.9990</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>responsable 3</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="57.6" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -6128,6 +6133,11 @@
       <c r="C18" s="6" t="inlineStr">
         <is>
           <t>41.1095, 16.8817</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>responsable 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
arrglos y nuevo elmento en popup: visualización del plan de estudios en erasmus out
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -5762,7 +5762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="11.44140625" customWidth="1" min="1" max="1"/>
@@ -5791,6 +5791,11 @@
           <t>responsable 1</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>https://radboud.nl/laura-TEST-EDITED</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
@@ -5813,6 +5818,11 @@
           <t>responsable 2</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://uniba.sk/pedro2</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="86.40000000000001" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -5835,6 +5845,11 @@
           <t>responsable 8</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://mdu.se/anna-nuevo-editado</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.6" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -5857,6 +5872,11 @@
           <t>responsable 5</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://agh.edu.pl/sofia</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -5874,6 +5894,11 @@
           <t>53.1325, 23.1688</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://pb.edu.pl/jean</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28.8" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -5896,6 +5921,11 @@
           <t>responsable 8</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://mdu.se/anna-nuevo-editado</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -5940,6 +5970,11 @@
           <t>responsable 8</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://mdu.se/anna-nuevo-editado</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.6" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -5962,6 +5997,11 @@
           <t>responsable 7</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>unop</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="57.6" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -5979,6 +6019,11 @@
           <t>46.5592, 15.6433</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://um.si/plan-test-xxx</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="57.6" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -6018,6 +6063,11 @@
           <t>responsable 2</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://uniba.sk/pedro2</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="43.2" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -6055,6 +6105,11 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>repsonsable 6</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://uno.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prueba de arreglos de MSIX (botón de segundo plano, e icono de escritorio con el icono de la aplicación)
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -5820,7 +5820,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://uniba.sk/pedro2</t>
+          <t>https://uniba.sk/pedro3</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://uniba.sk/pedro2</t>
+          <t>https://uniba.sk/pedro3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
la recarga del mapa optimizada solo carga el tipo de movilidad y curso academico actualizado
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -3691,17 +3691,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Alu. 90</t>
+          <t>Alu.</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Ape. 90</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Ape2. 90</t>
+          <t>Ape. 90 Ape2. 90</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -5376,6 +5381,7 @@
         </is>
       </c>
     </row>
+    <row r="150"/>
     <row r="151">
       <c r="O151" s="9" t="n"/>
     </row>

</xml_diff>

<commit_message>
refactor: eliminar código muerto de geocodificación y ampliar cobertura de tests
- Eliminadas _recalculate_coords, _recalculate_coords_ws y _geolocator de
  _excel_cells.py (nunca se invocaban; la geocodificación real vive en
  _coords_sheet.py)
- Limpiado import y __all__ en excel_update.py
- Añadidos 83 tests nuevos: test_excel_cells.py, test_loaders_common.py,
  test_api.py (total 211 tests, todos en verde)
- CI actualizado con --cov para generar informe de cobertura en cada push
- requirements-dev.txt unificado con requirements.txt vía -r y añadido
  pytest-cov con upper bounds
- README actulizado
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS OUT.xlsx
+++ b/install_root/data_demo/ERASMUS OUT.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,9 @@
       <u val="single"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -67,7 +70,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -120,12 +123,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -150,6 +159,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,76 +528,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O151"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:N150"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>apellido1</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>apellido2</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>curso</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>duracion meses</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>responsable programa</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="10" t="inlineStr">
         <is>
           <t>LA</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>Enlace plan de estudios</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="10" t="inlineStr">
         <is>
           <t>Destino</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>Ciudad</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
         <is>
           <t>País</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>ToR</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" s="10" t="inlineStr">
         <is>
           <t>Añade más campos que veas que hacen falta</t>
         </is>
@@ -607,7 +619,7 @@
           <t xml:space="preserve">Ape2. 1 </t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>alu1@correo.com</t>
         </is>
@@ -623,6 +635,7 @@
           <t>responsable 1</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>https://radboud.nl/laura</t>
@@ -648,6 +661,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -676,6 +690,7 @@
       <c r="F3" t="n">
         <v>5</v>
       </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>https://pedro-la.com</t>
@@ -706,6 +721,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -734,6 +750,7 @@
       <c r="F4" t="n">
         <v>2</v>
       </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>https://anna-la.com</t>
@@ -764,6 +781,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -792,6 +810,7 @@
       <c r="F5" t="n">
         <v>9</v>
       </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>https://sofia-la.com</t>
@@ -822,6 +841,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -850,6 +870,7 @@
       <c r="F6" t="n">
         <v>9</v>
       </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>https://jean-la.com</t>
@@ -880,6 +901,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -905,6 +927,8 @@
       <c r="E7" t="n">
         <v>3</v>
       </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>https://elena-la.ccom</t>
@@ -935,6 +959,7 @@
           <t>unamala.vom</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -963,6 +988,7 @@
       <c r="F8" t="n">
         <v>5</v>
       </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>https://marta-la.com</t>
@@ -993,6 +1019,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1021,6 +1048,8 @@
       <c r="F9" t="n">
         <v>9</v>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>https://radboud.nl/pablo</t>
@@ -1046,6 +1075,7 @@
           <t>unamala.vom</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1074,6 +1104,7 @@
       <c r="F10" t="n">
         <v>6</v>
       </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>https://carla-la.com</t>
@@ -1104,6 +1135,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1132,6 +1164,7 @@
       <c r="F11" t="n">
         <v>5</v>
       </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>https://diego-la.com</t>
@@ -1162,6 +1195,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1190,6 +1224,7 @@
       <c r="F12" t="n">
         <v>6</v>
       </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>https://valentina-la.com</t>
@@ -1220,6 +1255,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1248,6 +1284,7 @@
       <c r="F13" t="n">
         <v>5</v>
       </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>https://daniel-la.com</t>
@@ -1278,6 +1315,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1306,6 +1344,8 @@
       <c r="F14" t="n">
         <v>5</v>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>https://um.si/ana</t>
@@ -1331,6 +1371,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1353,6 +1394,9 @@
           <t>carla.oliveira@uclm.es</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://carla-la.com</t>
@@ -1378,6 +1422,8 @@
           <t>PAISES BAJOS</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1406,6 +1452,7 @@
       <c r="F16" t="n">
         <v>5</v>
       </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>https://ines-la.com</t>
@@ -1436,6 +1483,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1464,6 +1512,7 @@
       <c r="F17" t="n">
         <v>5</v>
       </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>https://samuel-la.com</t>
@@ -1494,6 +1543,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1522,6 +1572,7 @@
       <c r="F18" t="n">
         <v>5</v>
       </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>https://beatriz-la.com</t>
@@ -1552,6 +1603,7 @@
           <t>https://uclm.es/erasmus/ToR/2024-25/GomezLaura_Radboud_TOR_signed.pdf</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1574,16 +1626,13 @@
           <t>luca.rossi@uclm.es</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>TFG_MariaPicazoSanchez (2).pdf</t>
@@ -1609,6 +1658,8 @@
           <t>PAISES BAJOS</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1626,7 +1677,7 @@
           <t>Ape2. 19</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Pepu@alu.com</t>
         </is>
@@ -1637,6 +1688,8 @@
       <c r="F20" t="n">
         <v>5</v>
       </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>https://ku.lt/nuria</t>
@@ -1657,6 +1710,8 @@
           <t>PAISES BAJOS</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1674,21 +1729,29 @@
           <t>Ape2. 20</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>responsable 2</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1706,16 +1769,25 @@
           <t>Ape2. 21</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1733,16 +1805,25 @@
           <t>Ape2. 22</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1760,16 +1841,25 @@
           <t>Ape2. 23</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1787,16 +1877,25 @@
           <t>Ape2. 24</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1814,16 +1913,25 @@
           <t>Ape2. 25</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1841,16 +1949,25 @@
           <t>Ape2. 26</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1868,16 +1985,25 @@
           <t>Ape2. 27</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1895,16 +2021,25 @@
           <t>Ape2. 28</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1922,16 +2057,25 @@
           <t>Ape2. 29</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1949,16 +2093,25 @@
           <t>Ape2. 30</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1976,16 +2129,25 @@
           <t>Ape2. 31</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2003,16 +2165,25 @@
           <t>Ape2. 32</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2030,16 +2201,25 @@
           <t>Ape2. 33</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2057,21 +2237,29 @@
           <t>Ape2. 34</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>responsable 3</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2089,16 +2277,25 @@
           <t>Ape2. 35</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2116,16 +2313,25 @@
           <t>Ape2. 36</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2143,16 +2349,25 @@
           <t>Ape2. 37</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2170,16 +2385,25 @@
           <t>Ape2. 38</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2197,16 +2421,25 @@
           <t>Ape2. 39</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2224,16 +2457,25 @@
           <t>Ape2. 40</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2251,16 +2493,25 @@
           <t>Ape2. 41</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2278,16 +2529,25 @@
           <t>Ape2. 42</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2305,16 +2565,25 @@
           <t>Ape2. 43</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2332,16 +2601,25 @@
           <t>Ape2. 44</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2359,16 +2637,25 @@
           <t>Ape2. 45</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2386,16 +2673,25 @@
           <t>Ape2. 46</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2413,16 +2709,25 @@
           <t>Ape2. 47</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2440,16 +2745,25 @@
           <t>Ape2. 48</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2467,16 +2781,25 @@
           <t>Ape2. 49</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2494,16 +2817,25 @@
           <t>Ape2. 50</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2521,16 +2853,25 @@
           <t>Ape2. 51</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2548,16 +2889,25 @@
           <t>Ape2. 52</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2575,16 +2925,25 @@
           <t>Ape2. 53</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2602,16 +2961,25 @@
           <t>Ape2. 54</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2629,16 +2997,25 @@
           <t>Ape2. 55</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
           <t>University of Rzeszów</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2656,11 +3033,16 @@
           <t>Ape2. 56</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>responsable 4</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2676,6 +3058,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2693,6 +3077,12 @@
           <t>Ape2. 57</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2708,6 +3098,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2725,6 +3117,12 @@
           <t>Ape2. 58</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2740,6 +3138,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2757,6 +3157,12 @@
           <t>Ape2. 59</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2772,6 +3178,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2789,6 +3197,12 @@
           <t>Ape2. 60</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2804,6 +3218,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2821,6 +3237,12 @@
           <t>Ape2. 61</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2836,6 +3258,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2853,6 +3277,12 @@
           <t>Ape2. 62</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2868,6 +3298,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2885,6 +3317,12 @@
           <t>Ape2. 63</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2900,6 +3338,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2917,6 +3357,12 @@
           <t>Ape2. 64</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2932,6 +3378,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2949,6 +3397,12 @@
           <t>Ape2. 65</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2964,6 +3418,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2981,6 +3437,12 @@
           <t>Ape2. 66</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -2996,6 +3458,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3013,6 +3477,12 @@
           <t>Ape2. 67</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3028,6 +3498,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3045,6 +3517,12 @@
           <t>Ape2. 68</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3060,6 +3538,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3077,6 +3557,12 @@
           <t>Ape2. 69</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3092,6 +3578,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3109,6 +3597,12 @@
           <t>Ape2. 70</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3124,6 +3618,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3141,6 +3637,12 @@
           <t>Ape2. 71</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3156,6 +3658,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3173,6 +3677,12 @@
           <t>Ape2. 72</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3188,6 +3698,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3205,6 +3717,12 @@
           <t>Ape2. 73</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3220,6 +3738,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3237,6 +3757,12 @@
           <t>Ape2. 74</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3252,6 +3778,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3269,6 +3797,12 @@
           <t>Ape2. 75</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3284,6 +3818,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3301,6 +3837,12 @@
           <t>Ape2. 76</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3316,6 +3858,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3333,6 +3877,12 @@
           <t>Ape2. 77</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3348,6 +3898,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3365,6 +3917,12 @@
           <t>Ape2. 78</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3380,6 +3938,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3397,6 +3957,12 @@
           <t>Ape2. 79</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr">
         <is>
           <t>Università degli Studi di Bari Aldo Moro</t>
@@ -3412,6 +3978,8 @@
           <t>Italia</t>
         </is>
       </c>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3429,21 +3997,29 @@
           <t>Ape2. 80</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>responsable 5</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3461,16 +4037,25 @@
           <t>Ape2. 81</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3488,16 +4073,25 @@
           <t>Ape2. 82</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3515,16 +4109,25 @@
           <t>Ape2. 83</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3542,16 +4145,25 @@
           <t>Ape2. 84</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3569,16 +4181,25 @@
           <t>Ape2. 85</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3596,16 +4217,25 @@
           <t>Ape2. 86</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3623,16 +4253,25 @@
           <t>Ape2. 87</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3650,16 +4289,25 @@
           <t>Ape2. 88</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3677,16 +4325,25 @@
           <t>Ape2. 89</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
           <t>AGH University of Science and Technology</t>
         </is>
       </c>
+      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>POLONIA</t>
         </is>
       </c>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3704,16 +4361,18 @@
           <t>Ape. 90 Ape2. 90</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="n">
+        <v>3</v>
+      </c>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>repsonsable 6</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3729,6 +4388,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3746,6 +4407,12 @@
           <t>Ape2. 91</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3761,6 +4428,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3778,6 +4447,12 @@
           <t>Ape2. 92</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3793,6 +4468,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3810,6 +4487,12 @@
           <t>Ape2. 93</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3825,6 +4508,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3842,6 +4527,12 @@
           <t>Ape2. 94</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3857,6 +4548,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3874,6 +4567,12 @@
           <t>Ape2. 95</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3889,6 +4588,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3906,6 +4607,12 @@
           <t>Ape2. 96</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3921,6 +4628,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3938,6 +4647,12 @@
           <t>Ape2. 97</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3953,6 +4668,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3970,6 +4687,12 @@
           <t>Ape2. 98</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr">
         <is>
           <t>London University</t>
@@ -3985,6 +4708,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4002,6 +4727,12 @@
           <t>Ape2. 99</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr">
         <is>
           <t>London University</t>
@@ -4017,6 +4748,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4034,6 +4767,12 @@
           <t>Ape2. 100</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr">
         <is>
           <t>London University</t>
@@ -4049,6 +4788,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4066,6 +4807,12 @@
           <t>Ape2. 101</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr">
         <is>
           <t>London University</t>
@@ -4081,6 +4828,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4098,6 +4847,12 @@
           <t>Ape2. 102</t>
         </is>
       </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr">
         <is>
           <t>London University</t>
@@ -4113,6 +4868,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4130,6 +4887,12 @@
           <t>Ape2. 103</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
           <t>London University</t>
@@ -4145,6 +4908,8 @@
           <t>Reino Unido</t>
         </is>
       </c>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4162,21 +4927,29 @@
           <t>Ape2. 104</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>responsable 7</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4194,16 +4967,25 @@
           <t>Ape2. 105</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4221,16 +5003,25 @@
           <t>Ape2. 106</t>
         </is>
       </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4248,16 +5039,25 @@
           <t>Ape2. 107</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4275,16 +5075,25 @@
           <t>Ape2. 108</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4302,16 +5111,25 @@
           <t>Ape2. 109</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4329,16 +5147,25 @@
           <t>Ape2. 110</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4356,16 +5183,25 @@
           <t>Ape2. 111</t>
         </is>
       </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4383,16 +5219,25 @@
           <t>Ape2. 112</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4410,16 +5255,25 @@
           <t>Ape2. 113</t>
         </is>
       </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4437,16 +5291,25 @@
           <t>Ape2. 114</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4464,16 +5327,25 @@
           <t>Ape2. 115</t>
         </is>
       </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4491,16 +5363,25 @@
           <t>Ape2. 116</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4518,16 +5399,25 @@
           <t>Ape2. 117</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4545,16 +5435,25 @@
           <t>Ape2. 118</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4572,16 +5471,25 @@
           <t>Ape2. 119</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4599,16 +5507,25 @@
           <t>Ape2. 120</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4626,16 +5543,25 @@
           <t>Ape2. 121</t>
         </is>
       </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr">
         <is>
           <t>Universidade da Madeira</t>
         </is>
       </c>
+      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4658,21 +5584,28 @@
           <t>Alu122@correo.com</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>responsable 8</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
           <t>Suecia</t>
         </is>
       </c>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4690,16 +5623,25 @@
           <t>Ape2. 123</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4717,16 +5659,25 @@
           <t>Ape2. 124</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4744,16 +5695,25 @@
           <t>Ape2. 125</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4771,16 +5731,25 @@
           <t>Ape2. 126</t>
         </is>
       </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4798,16 +5767,25 @@
           <t>Ape2. 127</t>
         </is>
       </c>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4825,16 +5803,25 @@
           <t>Ape2. 128</t>
         </is>
       </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M129" t="inlineStr"/>
+      <c r="N129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4852,16 +5839,25 @@
           <t>Ape2. 129</t>
         </is>
       </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M130" t="inlineStr"/>
+      <c r="N130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4879,16 +5875,25 @@
           <t>Ape2. 130</t>
         </is>
       </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M131" t="inlineStr"/>
+      <c r="N131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4906,16 +5911,25 @@
           <t>Ape2. 131</t>
         </is>
       </c>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K132" t="inlineStr"/>
       <c r="L132" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M132" t="inlineStr"/>
+      <c r="N132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4933,16 +5947,25 @@
           <t>Ape2. 132</t>
         </is>
       </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M133" t="inlineStr"/>
+      <c r="N133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4960,16 +5983,25 @@
           <t>Ape2. 133</t>
         </is>
       </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M134" t="inlineStr"/>
+      <c r="N134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4987,16 +6019,25 @@
           <t>Ape2. 134</t>
         </is>
       </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5014,16 +6055,25 @@
           <t>Ape2. 135</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M136" t="inlineStr"/>
+      <c r="N136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5041,16 +6091,25 @@
           <t>Ape2. 136</t>
         </is>
       </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5068,16 +6127,25 @@
           <t>Ape2. 137</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M138" t="inlineStr"/>
+      <c r="N138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5095,16 +6163,25 @@
           <t>Ape2. 138</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
       <c r="J139" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5122,16 +6199,25 @@
           <t>Ape2. 139</t>
         </is>
       </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
       <c r="J140" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5149,16 +6235,25 @@
           <t>Ape2. 140</t>
         </is>
       </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5176,16 +6271,25 @@
           <t>Ape2. 141</t>
         </is>
       </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
       <c r="J142" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5203,16 +6307,25 @@
           <t>Ape2. 142</t>
         </is>
       </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
       <c r="J143" t="inlineStr">
         <is>
           <t>Mälardalen University</t>
         </is>
       </c>
+      <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr">
         <is>
           <t>SUECIA</t>
         </is>
       </c>
+      <c r="M143" t="inlineStr"/>
+      <c r="N143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5230,21 +6343,29 @@
           <t>Ape2. 143</t>
         </is>
       </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>responsable 9</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M144" t="inlineStr"/>
+      <c r="N144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5262,16 +6383,25 @@
           <t>Ape2. 144</t>
         </is>
       </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5289,16 +6419,25 @@
           <t>Ape2. 145</t>
         </is>
       </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
       <c r="J146" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5316,16 +6455,25 @@
           <t>Ape2. 146</t>
         </is>
       </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
       <c r="J147" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5343,16 +6491,25 @@
           <t>Ape2. 147</t>
         </is>
       </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
       <c r="J148" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
+      <c r="M148" t="inlineStr"/>
+      <c r="N148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5370,26 +6527,63 @@
           <t>Ape2. 148</t>
         </is>
       </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr">
         <is>
           <t>Comenius University in Bratislava</t>
         </is>
       </c>
+      <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr">
         <is>
           <t>REPÚBLICA ESLOVACA</t>
         </is>
       </c>
-    </row>
-    <row r="150"/>
-    <row r="151">
-      <c r="O151" s="9" t="n"/>
+      <c r="M149" t="inlineStr"/>
+      <c r="N149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Paco</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Pérez</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>responsable 8</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Mälardalen University</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Suecia</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr"/>
+      <c r="N150" t="inlineStr"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>